<commit_message>
revised details and recorded in md files
</commit_message>
<xml_diff>
--- a/output/reference_data/20260302_dashboards_ideas.xlsx
+++ b/output/reference_data/20260302_dashboards_ideas.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{910522C8-42EB-45D7-A60D-A7E4DAD5704D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atulvhanmarathi/projects/web_scrapping/output/reference_data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E68B00-2687-9E45-A9BE-33E8E2157DED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10935" yWindow="-10898" windowWidth="19395" windowHeight="10276" firstSheet="4" activeTab="6" xr2:uid="{0EDEF85B-854A-4C92-9982-68F507F89611}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18240" firstSheet="1" activeTab="4" xr2:uid="{0EDEF85B-854A-4C92-9982-68F507F89611}"/>
   </bookViews>
   <sheets>
     <sheet name="Aircraft Dim" sheetId="4" r:id="rId1"/>
     <sheet name="Trip Fact Table" sheetId="2" r:id="rId2"/>
     <sheet name="Booking Fact Table" sheetId="3" r:id="rId3"/>
     <sheet name="Utilization Visuals" sheetId="5" r:id="rId4"/>
-    <sheet name="Maintenance Jobs Fact " sheetId="9" r:id="rId5"/>
-    <sheet name="Maintenance Details Fact Table" sheetId="6" r:id="rId6"/>
-    <sheet name="Maintenance Visuals" sheetId="8" r:id="rId7"/>
+    <sheet name="Sheet1" sheetId="10" r:id="rId5"/>
+    <sheet name="Maintenance Jobs Fact " sheetId="9" r:id="rId6"/>
+    <sheet name="Maintenance Details Fact Table" sheetId="6" r:id="rId7"/>
+    <sheet name="Maintenance Visuals" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="157">
   <si>
     <t>Aircraft No</t>
   </si>
@@ -406,13 +412,115 @@
   </si>
   <si>
     <t>Front tyre</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> # </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> File Name                      </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Columns </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rows    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> What the data represents                                                                 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> dim_aircraft.csv               </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Master registry of all 62 aircraft — model, tail number, engine type, base facility, delivery date, range, and seat capacity </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> dim_airport.csv                </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Reference table for 34 airports — ICAO code, city, state, runway specs, and PC-12/PC-24 accessibility flags </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> dim_component.csv              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Aviation component catalogue with JASC/ATA codes and historical failure weight by model used to drive maintenance simulation </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> dim_crew.csv                   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Pilot and co-pilot roster — crew ID, role, home facility, and type ratings held </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> dim_date.csv                   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Full 3-year calendar spine (2023–2025) with day, week, month, quarter, season, holiday flags, and fiscal year </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> dim_facility.csv               </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Two maintenance facilities (Portsmouth NH and Boulder City NV) with technician count and bay capacity </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> dim_owner.csv                  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Fractional owner profiles — share type (1/8, 1/16, Cobalt), contracted hours, region, tenure, and aircraft preference </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fact_aircraft_daily_status.csv </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> One row per aircraft per calendar day — operational status (FLYING / AVAILABLE / IN_MAINTENANCE / AOG), flight hours, and cycles </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fact_booking.csv               </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Owner booking records — departure/destination, trip purpose, booking channel, passenger count, and lead time </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fact_flight.csv                </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Core flight ledger — every flight leg with origin/destination ICAO, hours, distance, fuel, passenger count, deadhead flag, and season </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fact_maintenance_detail.csv    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Line-item cost breakdown for each maintenance job — part/labor category, ATA code, quantity, unit cost, and extended cost </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fact_maintenance_job.csv       </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Maintenance job header — job type, severity, scheduled vs. unscheduled flag, start/close datetime, elapsed hours, and technician assigned </t>
+  </si>
+  <si>
+    <t xml:space="preserve">   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> **TOTAL**                      </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> **138** </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> **340,977** </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> **12 tables · 7 dimension + 5 fact · 3 years of simulated operations (Jan 2023 – Dec 2025)** </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -432,6 +540,13 @@
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -580,7 +695,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -591,6 +706,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -599,6 +720,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -609,27 +736,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -965,18 +1073,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB229DD4-DF91-4D28-925D-F3388AE6B394}">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="15.36328125" customWidth="1"/>
-    <col min="8" max="8" width="31.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.33203125" customWidth="1"/>
+    <col min="8" max="8" width="31.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1005,7 +1113,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -1016,7 +1124,7 @@
         <v>1995</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>41</v>
       </c>
@@ -1027,7 +1135,7 @@
         <v>2001</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -1038,7 +1146,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -1049,7 +1157,7 @@
         <v>2013</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>48</v>
       </c>
@@ -1060,7 +1168,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>49</v>
       </c>
@@ -1068,7 +1176,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>50</v>
       </c>
@@ -1076,7 +1184,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>51</v>
       </c>
@@ -1084,7 +1192,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>52</v>
       </c>
@@ -1092,7 +1200,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>53</v>
       </c>
@@ -1100,7 +1208,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -1111,7 +1219,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>54</v>
       </c>
@@ -1122,7 +1230,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>55</v>
       </c>
@@ -1133,7 +1241,7 @@
         <v>2022</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>56</v>
       </c>
@@ -1144,7 +1252,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>57</v>
       </c>
@@ -1164,18 +1272,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B42649B-7573-4EA4-BF81-EC0736FB6222}">
   <dimension ref="A1:N5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.6328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -1219,7 +1327,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>45658</v>
       </c>
@@ -1257,7 +1365,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>45658</v>
       </c>
@@ -1295,7 +1403,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>45667</v>
       </c>
@@ -1324,7 +1432,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>45672</v>
       </c>
@@ -1361,20 +1469,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5A125D8-7071-47BC-BFDE-D84EE4F34B0B}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="11.1796875" customWidth="1"/>
-    <col min="6" max="6" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7265625" customWidth="1"/>
-    <col min="8" max="8" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="11.1640625" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" customWidth="1"/>
+    <col min="8" max="8" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>26</v>
       </c>
@@ -1409,7 +1517,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>18</v>
       </c>
@@ -1417,7 +1525,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="I3" t="s">
         <v>37</v>
       </c>
@@ -1429,23 +1537,24 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE3B9442-D74C-494E-B718-2527E466EA85}">
-  <dimension ref="B2:K10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B2:V10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="2" max="2" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
+    <col min="20" max="20" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B3" s="10" t="s">
+    <row r="2" spans="2:22" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="2:22" x14ac:dyDescent="0.2">
+      <c r="B3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="12"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="14"/>
       <c r="G3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1455,8 +1564,23 @@
       <c r="K3" s="3" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="4" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M3" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="14"/>
+      <c r="R3" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="2:22" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>58</v>
       </c>
@@ -1468,9 +1592,20 @@
       <c r="G4" s="4"/>
       <c r="I4" s="4"/>
       <c r="K4" s="4"/>
-    </row>
-    <row r="5" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="M4" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="P4" s="9"/>
+      <c r="R4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="V4" s="4"/>
+    </row>
+    <row r="5" spans="2:22" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
         <v>61</v>
       </c>
@@ -1486,8 +1621,22 @@
         <v>64</v>
       </c>
       <c r="K6" s="6"/>
-    </row>
-    <row r="7" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="M6" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="N6" s="16"/>
+      <c r="P6" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="Q6" s="6"/>
+      <c r="S6" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="U6" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="2:22" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4"/>
       <c r="D7" s="7"/>
       <c r="E7" s="9"/>
@@ -1495,116 +1644,336 @@
       <c r="H7" s="9"/>
       <c r="J7" s="7"/>
       <c r="K7" s="9"/>
-    </row>
-    <row r="8" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="9" spans="2:11" ht="128.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="13" t="s">
+      <c r="M7" s="7"/>
+      <c r="N7" s="9"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="9"/>
+      <c r="S7" s="4"/>
+      <c r="U7" s="4"/>
+    </row>
+    <row r="8" spans="2:22" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="2:22" ht="128.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="15"/>
-      <c r="H9" s="13" t="s">
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="19"/>
+      <c r="H9" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="15"/>
-    </row>
-    <row r="10" spans="2:11" ht="115" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="13" t="s">
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="19"/>
+      <c r="M9" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="18"/>
+      <c r="Q9" s="19"/>
+      <c r="S9" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="T9" s="18"/>
+      <c r="U9" s="18"/>
+      <c r="V9" s="19"/>
+    </row>
+    <row r="10" spans="2:22" ht="115" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="15"/>
-      <c r="H10" s="16" t="s">
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="19"/>
+      <c r="H10" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="19"/>
+      <c r="M10" s="17" t="s">
+        <v>117</v>
+      </c>
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="18"/>
+      <c r="Q10" s="19"/>
+      <c r="S10" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="T10" s="18"/>
+      <c r="U10" s="18"/>
+      <c r="V10" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="11">
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="H9:K9"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="H10:K10"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="M9:Q9"/>
+    <mergeCell ref="S9:V9"/>
+    <mergeCell ref="M10:Q10"/>
+    <mergeCell ref="S10:V10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9CCDDE6-A66F-4663-ACA0-240564097940}">
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F17F4A59-7EF0-D14B-8F87-E4E2C8F6672E}">
+  <dimension ref="B1:F14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="105.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E1" t="s">
+        <v>126</v>
+      </c>
+      <c r="F1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D2">
+        <v>14</v>
+      </c>
+      <c r="E2">
+        <v>62</v>
+      </c>
+      <c r="F2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B3">
         <v>2</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="1">
-        <v>45667</v>
-      </c>
-      <c r="B2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="E3" t="s">
-        <v>106</v>
+      <c r="C3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3">
+        <v>11</v>
+      </c>
+      <c r="E3">
+        <v>34</v>
+      </c>
+      <c r="F3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4">
+        <v>6</v>
+      </c>
+      <c r="E4">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>120</v>
+      </c>
+      <c r="F5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6">
+        <v>14</v>
+      </c>
+      <c r="E6" s="20">
+        <v>1096</v>
+      </c>
+      <c r="F6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D7">
+        <v>7</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>140</v>
+      </c>
+      <c r="D8">
+        <v>13</v>
+      </c>
+      <c r="E8">
+        <v>350</v>
+      </c>
+      <c r="F8" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9" t="s">
+        <v>142</v>
+      </c>
+      <c r="D9">
+        <v>6</v>
+      </c>
+      <c r="E9" s="20">
+        <v>63080</v>
+      </c>
+      <c r="F9" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>144</v>
+      </c>
+      <c r="D10">
+        <v>13</v>
+      </c>
+      <c r="E10" s="20">
+        <v>124063</v>
+      </c>
+      <c r="F10" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>146</v>
+      </c>
+      <c r="D11">
+        <v>26</v>
+      </c>
+      <c r="E11" s="20">
+        <v>143039</v>
+      </c>
+      <c r="F11" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>148</v>
+      </c>
+      <c r="D12">
+        <v>13</v>
+      </c>
+      <c r="E12" s="20">
+        <v>6626</v>
+      </c>
+      <c r="F12" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>150</v>
+      </c>
+      <c r="D13">
+        <v>16</v>
+      </c>
+      <c r="E13" s="20">
+        <v>2485</v>
+      </c>
+      <c r="F13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>152</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="D14" s="21" t="s">
+        <v>154</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="F14" s="21" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -1613,24 +1982,20 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{587249FA-6B54-4D67-8259-8CE11835FB6F}">
-  <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9CCDDE6-A66F-4663-ACA0-240564097940}">
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.26953125" customWidth="1"/>
-    <col min="6" max="6" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8" style="21" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7265625" style="21"/>
-    <col min="11" max="11" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
@@ -1644,28 +2009,25 @@
         <v>83</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="I1" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="J1" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+        <v>109</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>45667</v>
       </c>
@@ -1679,364 +2041,12 @@
         <v>79</v>
       </c>
       <c r="E2" t="s">
-        <v>91</v>
-      </c>
-      <c r="F2" t="s">
-        <v>86</v>
-      </c>
-      <c r="H2" t="s">
-        <v>96</v>
-      </c>
-      <c r="I2" s="21">
-        <v>5</v>
-      </c>
-      <c r="J2" s="21">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" s="1">
-        <v>45667</v>
-      </c>
-      <c r="B3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D3" t="s">
-        <v>79</v>
-      </c>
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="E3" t="s">
-        <v>90</v>
-      </c>
-      <c r="F3" t="s">
-        <v>86</v>
-      </c>
-      <c r="H3" t="s">
-        <v>96</v>
-      </c>
-      <c r="I3" s="21">
-        <v>20</v>
-      </c>
-      <c r="J3" s="21">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="1">
-        <v>45667</v>
-      </c>
-      <c r="B4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D4" t="s">
-        <v>79</v>
-      </c>
-      <c r="E4" t="s">
-        <v>90</v>
-      </c>
-      <c r="F4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" t="s">
-        <v>121</v>
-      </c>
-      <c r="H4" t="s">
-        <v>93</v>
-      </c>
-      <c r="I4" s="21">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="1">
-        <v>45667</v>
-      </c>
-      <c r="B5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D5" t="s">
-        <v>79</v>
-      </c>
-      <c r="E5" t="s">
-        <v>90</v>
-      </c>
-      <c r="F5" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" t="s">
-        <v>122</v>
-      </c>
-      <c r="H5" t="s">
-        <v>93</v>
-      </c>
-      <c r="I5" s="21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" s="1">
-        <v>45667</v>
-      </c>
-      <c r="B6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D6" t="s">
-        <v>79</v>
-      </c>
-      <c r="E6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F6" t="s">
-        <v>87</v>
-      </c>
-      <c r="G6" t="s">
-        <v>100</v>
-      </c>
-      <c r="H6" t="s">
-        <v>93</v>
-      </c>
-      <c r="I6" s="21">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A7" s="1">
-        <v>45667</v>
-      </c>
-      <c r="B7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" t="s">
-        <v>80</v>
-      </c>
-      <c r="D7" t="s">
-        <v>79</v>
-      </c>
-      <c r="E7" t="s">
-        <v>91</v>
-      </c>
-      <c r="F7" t="s">
-        <v>87</v>
-      </c>
-      <c r="G7" t="s">
-        <v>101</v>
-      </c>
-      <c r="H7" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" s="1">
-        <v>45667</v>
-      </c>
-      <c r="B8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" t="s">
-        <v>80</v>
-      </c>
-      <c r="D8" t="s">
-        <v>79</v>
-      </c>
-      <c r="E8" t="s">
-        <v>86</v>
-      </c>
-      <c r="F8" t="s">
-        <v>88</v>
-      </c>
-      <c r="H8" t="s">
-        <v>96</v>
-      </c>
-      <c r="I8" s="21">
-        <v>5</v>
-      </c>
-      <c r="J8" s="21">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" s="1">
-        <v>45667</v>
-      </c>
-      <c r="B9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E9" t="s">
-        <v>114</v>
-      </c>
-      <c r="F9" t="s">
-        <v>114</v>
-      </c>
-      <c r="H9" t="s">
-        <v>115</v>
-      </c>
-      <c r="I9" s="21">
-        <v>400</v>
-      </c>
-      <c r="J9" s="21">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A10" s="1">
-        <v>45698</v>
-      </c>
-      <c r="B10" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" t="s">
-        <v>99</v>
-      </c>
-      <c r="E10" t="s">
-        <v>90</v>
-      </c>
-      <c r="F10" t="s">
-        <v>87</v>
-      </c>
-      <c r="G10" t="s">
-        <v>98</v>
-      </c>
-      <c r="H10" t="s">
-        <v>93</v>
-      </c>
-      <c r="I10" s="21">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A11" s="1">
-        <v>45698</v>
-      </c>
-      <c r="B11" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" t="s">
-        <v>81</v>
-      </c>
-      <c r="D11" t="s">
-        <v>99</v>
-      </c>
-      <c r="E11" t="s">
-        <v>90</v>
-      </c>
-      <c r="F11" t="s">
-        <v>87</v>
-      </c>
-      <c r="G11" t="s">
-        <v>97</v>
-      </c>
-      <c r="H11" t="s">
-        <v>93</v>
-      </c>
-      <c r="I11" s="21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" s="1">
-        <v>45698</v>
-      </c>
-      <c r="B12" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" t="s">
-        <v>81</v>
-      </c>
-      <c r="D12" t="s">
-        <v>99</v>
-      </c>
-      <c r="E12" t="s">
-        <v>114</v>
-      </c>
-      <c r="F12" t="s">
-        <v>114</v>
-      </c>
-      <c r="H12" t="s">
-        <v>115</v>
-      </c>
-      <c r="I12" s="21">
-        <v>800</v>
-      </c>
-      <c r="J12" s="21">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A13" s="1">
-        <v>45701</v>
-      </c>
-      <c r="B13" t="s">
-        <v>118</v>
-      </c>
-      <c r="C13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D13" t="s">
-        <v>119</v>
-      </c>
-      <c r="E13" t="s">
-        <v>120</v>
-      </c>
-      <c r="F13" t="s">
-        <v>86</v>
-      </c>
-      <c r="H13" t="s">
-        <v>96</v>
-      </c>
-      <c r="I13" s="21">
-        <v>20</v>
-      </c>
-      <c r="J13" s="21">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A14" s="1">
-        <v>45701</v>
-      </c>
-      <c r="B14" t="s">
-        <v>118</v>
-      </c>
-      <c r="C14" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" t="s">
-        <v>119</v>
-      </c>
-      <c r="E14" t="s">
-        <v>114</v>
-      </c>
-      <c r="F14" t="s">
-        <v>114</v>
-      </c>
-      <c r="H14" t="s">
-        <v>115</v>
-      </c>
-      <c r="I14" s="21">
-        <v>800</v>
-      </c>
-      <c r="J14" s="21">
-        <v>7</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -2045,25 +2055,457 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{587249FA-6B54-4D67-8259-8CE11835FB6F}">
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.6640625" style="10"/>
+    <col min="11" max="11" width="12.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>45667</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F2" t="s">
+        <v>86</v>
+      </c>
+      <c r="H2" t="s">
+        <v>96</v>
+      </c>
+      <c r="I2" s="10">
+        <v>5</v>
+      </c>
+      <c r="J2" s="10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>45667</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F3" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" t="s">
+        <v>96</v>
+      </c>
+      <c r="I3" s="10">
+        <v>20</v>
+      </c>
+      <c r="J3" s="10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>45667</v>
+      </c>
+      <c r="B4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" t="s">
+        <v>121</v>
+      </c>
+      <c r="H4" t="s">
+        <v>93</v>
+      </c>
+      <c r="I4" s="10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>45667</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F5" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" t="s">
+        <v>122</v>
+      </c>
+      <c r="H5" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>45667</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" t="s">
+        <v>90</v>
+      </c>
+      <c r="F6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G6" t="s">
+        <v>100</v>
+      </c>
+      <c r="H6" t="s">
+        <v>93</v>
+      </c>
+      <c r="I6" s="10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>45667</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E7" t="s">
+        <v>91</v>
+      </c>
+      <c r="F7" t="s">
+        <v>87</v>
+      </c>
+      <c r="G7" t="s">
+        <v>101</v>
+      </c>
+      <c r="H7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>45667</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F8" t="s">
+        <v>88</v>
+      </c>
+      <c r="H8" t="s">
+        <v>96</v>
+      </c>
+      <c r="I8" s="10">
+        <v>5</v>
+      </c>
+      <c r="J8" s="10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>45667</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" t="s">
+        <v>114</v>
+      </c>
+      <c r="F9" t="s">
+        <v>114</v>
+      </c>
+      <c r="H9" t="s">
+        <v>115</v>
+      </c>
+      <c r="I9" s="10">
+        <v>400</v>
+      </c>
+      <c r="J9" s="10">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>45698</v>
+      </c>
+      <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" t="s">
+        <v>90</v>
+      </c>
+      <c r="F10" t="s">
+        <v>87</v>
+      </c>
+      <c r="G10" t="s">
+        <v>98</v>
+      </c>
+      <c r="H10" t="s">
+        <v>93</v>
+      </c>
+      <c r="I10" s="10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>45698</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" t="s">
+        <v>81</v>
+      </c>
+      <c r="D11" t="s">
+        <v>99</v>
+      </c>
+      <c r="E11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" t="s">
+        <v>87</v>
+      </c>
+      <c r="G11" t="s">
+        <v>97</v>
+      </c>
+      <c r="H11" t="s">
+        <v>93</v>
+      </c>
+      <c r="I11" s="10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>45698</v>
+      </c>
+      <c r="B12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" t="s">
+        <v>99</v>
+      </c>
+      <c r="E12" t="s">
+        <v>114</v>
+      </c>
+      <c r="F12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H12" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" s="10">
+        <v>800</v>
+      </c>
+      <c r="J12" s="10">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>45701</v>
+      </c>
+      <c r="B13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E13" t="s">
+        <v>120</v>
+      </c>
+      <c r="F13" t="s">
+        <v>86</v>
+      </c>
+      <c r="H13" t="s">
+        <v>96</v>
+      </c>
+      <c r="I13" s="10">
+        <v>20</v>
+      </c>
+      <c r="J13" s="10">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>45701</v>
+      </c>
+      <c r="B14" t="s">
+        <v>118</v>
+      </c>
+      <c r="C14" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" t="s">
+        <v>119</v>
+      </c>
+      <c r="E14" t="s">
+        <v>114</v>
+      </c>
+      <c r="F14" t="s">
+        <v>114</v>
+      </c>
+      <c r="H14" t="s">
+        <v>115</v>
+      </c>
+      <c r="I14" s="10">
+        <v>800</v>
+      </c>
+      <c r="J14" s="10">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9F6A38B-0437-4046-A765-BCDE4F6B3816}">
   <dimension ref="B2:K10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.08984375" customWidth="1"/>
-    <col min="11" max="11" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.1640625" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B3" s="10" t="s">
+    <row r="2" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="12"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="14"/>
       <c r="G3" s="3" t="s">
         <v>82</v>
       </c>
@@ -2074,7 +2516,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>58</v>
       </c>
@@ -2087,12 +2529,12 @@
       <c r="I4" s="4"/>
       <c r="K4" s="4"/>
     </row>
-    <row r="5" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="6" spans="2:11" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="19" t="s">
+    <row r="5" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="6" spans="2:11" ht="29" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="20"/>
+      <c r="C6" s="16"/>
       <c r="E6" s="5" t="s">
         <v>74</v>
       </c>
@@ -2104,7 +2546,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B7" s="7"/>
       <c r="C7" s="9"/>
       <c r="E7" s="7"/>
@@ -2112,36 +2554,36 @@
       <c r="H7" s="4"/>
       <c r="J7" s="4"/>
     </row>
-    <row r="8" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="9" spans="2:11" ht="128.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="13" t="s">
+    <row r="8" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="2:11" ht="128.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="15"/>
-      <c r="H9" s="13" t="s">
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="19"/>
+      <c r="H9" s="17" t="s">
         <v>113</v>
       </c>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="15"/>
-    </row>
-    <row r="10" spans="2:11" ht="115" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="13" t="s">
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="19"/>
+    </row>
+    <row r="10" spans="2:11" ht="115" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="15"/>
-      <c r="H10" s="16" t="s">
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="19"/>
+      <c r="H10" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>